<commit_message>
Functional corrected simulator structure. Still requires a few additions
</commit_message>
<xml_diff>
--- a/legacy/activeDrag_mach_cd_Comp.xlsx
+++ b/legacy/activeDrag_mach_cd_Comp.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programming\Code\Code Projects\Python\Active Drag\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rex\Documents\GitHub\Active_Drag_2024_2026\legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{496B5108-E575-4119-AF99-648CC6B226BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9469494C-68BF-4D91-A18E-770B7D8AA5EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-2775" windowWidth="38640" windowHeight="23640" xr2:uid="{5885C0A6-86B6-40A2-80E4-D5A5D9881E2D}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{5885C0A6-86B6-40A2-80E4-D5A5D9881E2D}"/>
   </bookViews>
   <sheets>
     <sheet name="calculated" sheetId="1" r:id="rId1"/>
     <sheet name="rasaero values" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -257,7 +256,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -762,12 +761,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -938,7 +948,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -948,19 +957,28 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1031,10 +1049,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>calculated!$B$10:$B$15</c:f>
+              <c:f>calculated!$B$10:$B$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>0.2</c:v>
                 </c:pt>
@@ -1045,40 +1063,64 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.4</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.6</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>calculated!$D$10:$D$15</c:f>
+              <c:f>calculated!$D$10:$D$19</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0.52800000000000002</c:v>
+                  <c:v>0.47</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.52200000000000002</c:v>
+                  <c:v>0.47</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.53300000000000003</c:v>
+                  <c:v>0.47</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.54800000000000004</c:v>
+                  <c:v>0.47</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.67200000000000004</c:v>
+                  <c:v>0.63</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.70299999999999996</c:v>
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.56000000000000005</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.45</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1121,10 +1163,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>calculated!$B$10:$B$15</c:f>
+              <c:f>calculated!$B$10:$B$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>0.2</c:v>
                 </c:pt>
@@ -1135,40 +1177,64 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.4</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.6</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>calculated!$H$10:$H$15</c:f>
+              <c:f>calculated!$H$10:$H$19</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0.60077879236444953</c:v>
+                  <c:v>0.80958909378646138</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.59698386718486507</c:v>
+                  <c:v>0.81987807132605006</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.61177588118659387</c:v>
+                  <c:v>0.83757177792156701</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.63233371621683643</c:v>
+                  <c:v>0.87992140555247178</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.76391475198773817</c:v>
+                  <c:v>1.0588783355571327</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.80486148371278865</c:v>
+                  <c:v>1.0752902297767035</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.094773588881284</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.1098399411706557</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.1535276769380436</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.2194542445644689</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1210,10 +1276,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>calculated!$B$10:$B$15</c:f>
+              <c:f>calculated!$B$10:$B$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>0.2</c:v>
                 </c:pt>
@@ -1224,40 +1290,64 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.4</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.6</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>calculated!$L$10:$L$15</c:f>
+              <c:f>calculated!$L$10:$L$19</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0.80919566060380577</c:v>
+                  <c:v>1.149178187572923</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.81171541547556214</c:v>
+                  <c:v>1.1697561426521002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.83736663250724042</c:v>
+                  <c:v>1.2051435558431343</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.87384045808310185</c:v>
+                  <c:v>1.2898428111049438</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0271313310476431</c:v>
+                  <c:v>1.4877566711142658</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0965625512892234</c:v>
+                  <c:v>1.5505804595534074</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.6295471777625679</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.7196798823413117</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.8570553538760872</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.0389084891289384</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1333,7 +1423,7 @@
                         <c:v>0.6</c:v>
                       </c:pt>
                       <c:pt idx="3">
-                        <c:v>0.8</c:v>
+                        <c:v>0.9</c:v>
                       </c:pt>
                       <c:pt idx="4">
                         <c:v>1</c:v>
@@ -1354,25 +1444,25 @@
                       </c:ext>
                     </c:extLst>
                     <c:numCache>
-                      <c:formatCode>0.000</c:formatCode>
+                      <c:formatCode>General</c:formatCode>
                       <c:ptCount val="6"/>
                       <c:pt idx="0">
-                        <c:v>4.754598981227951</c:v>
+                        <c:v>18.857395415104982</c:v>
                       </c:pt>
                       <c:pt idx="1">
-                        <c:v>19.59462128694738</c:v>
+                        <c:v>77.714970931527219</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>46.317469834284111</c:v>
+                        <c:v>183.70147445467921</c:v>
                       </c:pt>
                       <c:pt idx="3">
-                        <c:v>88.151614102044775</c:v>
+                        <c:v>460.94976559879348</c:v>
                       </c:pt>
                       <c:pt idx="4">
-                        <c:v>150.11852078153987</c:v>
+                        <c:v>595.39076096319559</c:v>
                       </c:pt>
                       <c:pt idx="5">
-                        <c:v>239.56399487133484</c:v>
+                        <c:v>950.14384942811773</c:v>
                       </c:pt>
                     </c:numCache>
                   </c:numRef>
@@ -1436,7 +1526,7 @@
                         <c:v>0.6</c:v>
                       </c:pt>
                       <c:pt idx="3">
-                        <c:v>0.8</c:v>
+                        <c:v>0.9</c:v>
                       </c:pt>
                       <c:pt idx="4">
                         <c:v>1</c:v>
@@ -1522,7 +1612,7 @@
                         <c:v>0.6</c:v>
                       </c:pt>
                       <c:pt idx="3">
-                        <c:v>0.8</c:v>
+                        <c:v>0.9</c:v>
                       </c:pt>
                       <c:pt idx="4">
                         <c:v>1</c:v>
@@ -1607,7 +1697,7 @@
                         <c:v>0.6</c:v>
                       </c:pt>
                       <c:pt idx="3">
-                        <c:v>0.8</c:v>
+                        <c:v>0.9</c:v>
                       </c:pt>
                       <c:pt idx="4">
                         <c:v>1</c:v>
@@ -1693,7 +1783,7 @@
                         <c:v>0.6</c:v>
                       </c:pt>
                       <c:pt idx="3">
-                        <c:v>0.8</c:v>
+                        <c:v>0.9</c:v>
                       </c:pt>
                       <c:pt idx="4">
                         <c:v>1</c:v>
@@ -1778,7 +1868,7 @@
                         <c:v>0.6</c:v>
                       </c:pt>
                       <c:pt idx="3">
-                        <c:v>0.8</c:v>
+                        <c:v>0.9</c:v>
                       </c:pt>
                       <c:pt idx="4">
                         <c:v>1</c:v>
@@ -2013,7 +2103,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2095,6 +2185,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2102,7 +2193,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2201,7 +2291,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -2216,25 +2306,25 @@
             <c:numRef>
               <c:f>calculated!$D$10:$D$15</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.52800000000000002</c:v>
+                  <c:v>0.47</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.52200000000000002</c:v>
+                  <c:v>0.47</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.53300000000000003</c:v>
+                  <c:v>0.47</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.54800000000000004</c:v>
+                  <c:v>0.47</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.67200000000000004</c:v>
+                  <c:v>0.63</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.70299999999999996</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2291,7 +2381,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -2309,22 +2399,22 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.60077879236444953</c:v>
+                  <c:v>0.80958909378646138</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.59698386718486507</c:v>
+                  <c:v>0.81987807132605006</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.61177588118659387</c:v>
+                  <c:v>0.83757177792156701</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.63233371621683643</c:v>
+                  <c:v>0.87992140555247178</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.76391475198773817</c:v>
+                  <c:v>1.0588783355571327</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.80486148371278865</c:v>
+                  <c:v>1.0752902297767035</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2380,7 +2470,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -2398,22 +2488,22 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.80919566060380577</c:v>
+                  <c:v>1.149178187572923</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.81171541547556214</c:v>
+                  <c:v>1.1697561426521002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.83736663250724042</c:v>
+                  <c:v>1.2051435558431343</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.87384045808310185</c:v>
+                  <c:v>1.2898428111049438</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0271313310476431</c:v>
+                  <c:v>1.4877566711142658</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0965625512892234</c:v>
+                  <c:v>1.5505804595534074</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2470,7 +2560,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -2485,25 +2575,25 @@
             <c:numRef>
               <c:f>calculated!$P$10:$P$15</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>4.754598981227951</c:v>
+                  <c:v>18.857395415104982</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>19.59462128694738</c:v>
+                  <c:v>77.714970931527219</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>46.317469834284111</c:v>
+                  <c:v>183.70147445467921</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>88.151614102044775</c:v>
+                  <c:v>460.94976559879348</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>150.11852078153987</c:v>
+                  <c:v>595.39076096319559</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>239.56399487133484</c:v>
+                  <c:v>950.14384942811773</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2559,7 +2649,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -2631,7 +2721,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -2702,7 +2792,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -2774,7 +2864,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -2845,7 +2935,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.8</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -3081,7 +3171,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3163,6 +3253,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3170,7 +3261,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4321,16 +4411,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>419100</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>428625</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4718,7 +4808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC9E6B00-D973-480A-A161-3B0332E4ED97}">
-  <dimension ref="B1:AL19"/>
+  <dimension ref="B1:AL25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="10" max="10" width="8.85546875" customWidth="1"/>
@@ -4734,21 +4824,21 @@
   <sheetData>
     <row r="1" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="61"/>
-      <c r="J2" s="64" t="s">
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="60"/>
+      <c r="J2" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="65"/>
-      <c r="L2" s="65"/>
-      <c r="M2" s="66"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="63"/>
     </row>
     <row r="3" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -4825,18 +4915,18 @@
         <v>1.42</v>
       </c>
       <c r="N4" s="53">
-        <v>57205.800999999999</v>
+        <v>101325</v>
       </c>
       <c r="O4" s="53">
         <v>1.4</v>
       </c>
       <c r="P4">
-        <f>4*1.6*2.75</f>
-        <v>17.600000000000001</v>
+        <f>4*2*3</f>
+        <v>24</v>
       </c>
       <c r="Q4">
         <f>P4/1550</f>
-        <v>1.135483870967742E-2</v>
+        <v>1.5483870967741935E-2</v>
       </c>
     </row>
     <row r="5" spans="2:38" x14ac:dyDescent="0.25">
@@ -4889,91 +4979,94 @@
       <c r="N6" s="53">
         <v>101325</v>
       </c>
+      <c r="O6">
+        <v>57205</v>
+      </c>
     </row>
     <row r="7" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="59" t="s">
+      <c r="C8" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="59" t="s">
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="60"/>
+      <c r="G8" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="60"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="59" t="s">
+      <c r="H8" s="59"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="60"/>
+      <c r="K8" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="L8" s="60"/>
-      <c r="M8" s="60"/>
-      <c r="N8" s="61"/>
-      <c r="O8" s="59"/>
-      <c r="P8" s="60"/>
-      <c r="Q8" s="60"/>
-      <c r="R8" s="61"/>
-      <c r="S8" s="59"/>
-      <c r="T8" s="60"/>
-      <c r="U8" s="60"/>
-      <c r="V8" s="61"/>
-      <c r="W8" s="59"/>
-      <c r="X8" s="60"/>
-      <c r="Y8" s="60"/>
-      <c r="Z8" s="61"/>
-      <c r="AA8" s="64"/>
-      <c r="AB8" s="65"/>
-      <c r="AC8" s="65"/>
-      <c r="AD8" s="66"/>
-      <c r="AE8" s="64"/>
-      <c r="AF8" s="65"/>
-      <c r="AG8" s="65"/>
-      <c r="AH8" s="66"/>
-      <c r="AI8" s="59"/>
-      <c r="AJ8" s="60"/>
-      <c r="AK8" s="60"/>
-      <c r="AL8" s="61"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
+      <c r="N8" s="60"/>
+      <c r="O8" s="58"/>
+      <c r="P8" s="59"/>
+      <c r="Q8" s="59"/>
+      <c r="R8" s="60"/>
+      <c r="S8" s="58"/>
+      <c r="T8" s="59"/>
+      <c r="U8" s="59"/>
+      <c r="V8" s="60"/>
+      <c r="W8" s="58"/>
+      <c r="X8" s="59"/>
+      <c r="Y8" s="59"/>
+      <c r="Z8" s="60"/>
+      <c r="AA8" s="61"/>
+      <c r="AB8" s="62"/>
+      <c r="AC8" s="62"/>
+      <c r="AD8" s="63"/>
+      <c r="AE8" s="61"/>
+      <c r="AF8" s="62"/>
+      <c r="AG8" s="62"/>
+      <c r="AH8" s="63"/>
+      <c r="AI8" s="58"/>
+      <c r="AJ8" s="59"/>
+      <c r="AK8" s="59"/>
+      <c r="AL8" s="60"/>
     </row>
     <row r="9" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="63"/>
+      <c r="B9" s="65"/>
       <c r="C9" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="25" t="s">
+      <c r="G9" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="26" t="s">
+      <c r="H9" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="26" t="s">
+      <c r="I9" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="27" t="s">
+      <c r="J9" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="25" t="s">
+      <c r="K9" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="L9" s="26" t="s">
+      <c r="L9" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="M9" s="26" t="s">
+      <c r="M9" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="N9" s="27" t="s">
+      <c r="N9" s="48" t="s">
         <v>16</v>
       </c>
       <c r="O9" s="46"/>
@@ -5009,70 +5102,70 @@
       <c r="AK9" s="26"/>
       <c r="AL9" s="27"/>
     </row>
-    <row r="10" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B10" s="54">
         <v>0.2</v>
       </c>
       <c r="C10" s="57">
-        <f t="shared" ref="C10:C19" si="0">$N$4*((1+(($O$4-1)/2)*($B10^2))^($O$4/($O$4-1))) - $N$4</f>
-        <v>1617.8441867964648</v>
-      </c>
-      <c r="D10" s="34">
-        <v>0.52800000000000002</v>
-      </c>
-      <c r="E10" s="34">
+        <f>$N$4*((1+(($O$4-1)/2)*($B10^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>2865.5845973934047</v>
+      </c>
+      <c r="D10" s="57">
+        <v>0.47</v>
+      </c>
+      <c r="E10" s="35">
         <v>1.68</v>
       </c>
-      <c r="F10" s="39">
-        <f t="shared" ref="F10:F15" si="1">(E10-$M$4)/$L$4</f>
+      <c r="F10" s="68">
+        <f t="shared" ref="F10:F15" si="0">(E10-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G10" s="31">
-        <v>15</v>
-      </c>
-      <c r="H10" s="34">
-        <f t="shared" ref="H10:H19" si="2">$D10+( (0.85*$C10*$Q$4*SIN(RADIANS($G$10))) / (0.5*$K$4*(($B10*$J$4)^2)*PI()*((0.5*$L$4)^2)) )</f>
-        <v>0.60077879236444953</v>
-      </c>
-      <c r="I10" s="34">
+      <c r="G10" s="10">
+        <v>30</v>
+      </c>
+      <c r="H10" s="35">
+        <f t="shared" ref="H10:H19" si="1">$D10+( (0.85*$C10*$Q$4*SIN(RADIANS($G$10))) / (0.5*$K$4*(($B10*$J$4)^2)*PI()*((0.5*$L$4)^2)) )</f>
+        <v>0.80958909378646138</v>
+      </c>
+      <c r="I10" s="35">
         <v>1.68</v>
       </c>
-      <c r="J10" s="39">
-        <f t="shared" ref="J10:J15" si="3">(I10-$M$4)/$L$4</f>
+      <c r="J10" s="68">
+        <f t="shared" ref="J10:J15" si="2">(I10-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K10" s="31">
+      <c r="K10" s="10">
         <v>90</v>
       </c>
-      <c r="L10" s="34">
-        <f t="shared" ref="L10:L19" si="4">$D10+( (0.85*$C10*$Q$4*SIN(RADIANS($K$10))) / (0.5*$K$4*(($B10*$J$4)^2)*PI()*((0.5*$L$4)^2)) )</f>
-        <v>0.80919566060380577</v>
-      </c>
-      <c r="M10" s="34">
+      <c r="L10" s="35">
+        <f t="shared" ref="L10:L19" si="3">$D10+( (0.85*$C10*$Q$4*SIN(RADIANS($K$10))) / (0.5*$K$4*(($B10*$J$4)^2)*PI()*((0.5*$L$4)^2)) )</f>
+        <v>1.149178187572923</v>
+      </c>
+      <c r="M10" s="35">
         <v>1.68</v>
       </c>
-      <c r="N10" s="42">
-        <f t="shared" ref="N10:N15" si="5">(M10-$M$4)/$L$4</f>
+      <c r="N10" s="68">
+        <f t="shared" ref="N10:N15" si="4">(M10-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="O10" s="37"/>
-      <c r="P10" s="38">
-        <f t="shared" ref="P10:P19" si="6">$Q$4*SIN(RADIANS($G$10))*C10</f>
-        <v>4.754598981227951</v>
-      </c>
-      <c r="Q10" s="38">
-        <f>$Q$4*$C10</f>
-        <v>18.370359798463085</v>
-      </c>
-      <c r="R10">
+      <c r="O10" s="10"/>
+      <c r="P10" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C10)*0.85</f>
+        <v>18.857395415104982</v>
+      </c>
+      <c r="Q10" s="57">
+        <f>($Q$4*$C10)*0.85</f>
+        <v>37.714790830209971</v>
+      </c>
+      <c r="R10" s="57">
         <f>P10/4.448</f>
-        <v>1.0689296270746291</v>
-      </c>
-      <c r="S10" s="40">
+        <v>4.2395223505182056</v>
+      </c>
+      <c r="S10" s="68">
         <f>Q10/4.448</f>
-        <v>4.1300269331077075</v>
-      </c>
-      <c r="T10" s="34"/>
+        <v>8.4790447010364129</v>
+      </c>
+      <c r="T10" s="66"/>
       <c r="U10" s="34"/>
       <c r="V10" s="39"/>
       <c r="W10" s="31"/>
@@ -5092,66 +5185,66 @@
       <c r="AK10" s="34"/>
       <c r="AL10" s="39"/>
     </row>
-    <row r="11" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B11" s="55">
         <v>0.4</v>
       </c>
       <c r="C11" s="57">
+        <f>$N$4*((1+(($O$4-1)/2)*($B11^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>11809.627935673256</v>
+      </c>
+      <c r="D11" s="57">
+        <v>0.47</v>
+      </c>
+      <c r="E11" s="35">
+        <v>1.68</v>
+      </c>
+      <c r="F11" s="68">
         <f t="shared" si="0"/>
-        <v>6667.4485622715511</v>
-      </c>
-      <c r="D11" s="34">
-        <v>0.52200000000000002</v>
-      </c>
-      <c r="E11" s="34">
+        <v>1.6455696202531647</v>
+      </c>
+      <c r="G11" s="10"/>
+      <c r="H11" s="35">
+        <f t="shared" si="1"/>
+        <v>0.81987807132605006</v>
+      </c>
+      <c r="I11" s="35">
         <v>1.68</v>
       </c>
-      <c r="F11" s="39">
-        <f t="shared" si="1"/>
+      <c r="J11" s="68">
+        <f t="shared" si="2"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G11" s="32"/>
-      <c r="H11" s="34">
-        <f t="shared" si="2"/>
-        <v>0.59698386718486507</v>
-      </c>
-      <c r="I11" s="34">
+      <c r="K11" s="10"/>
+      <c r="L11" s="35">
+        <f t="shared" si="3"/>
+        <v>1.1697561426521002</v>
+      </c>
+      <c r="M11" s="35">
         <v>1.68</v>
       </c>
-      <c r="J11" s="39">
-        <f t="shared" si="3"/>
+      <c r="N11" s="68">
+        <f t="shared" si="4"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K11" s="32"/>
-      <c r="L11" s="34">
-        <f t="shared" si="4"/>
-        <v>0.81171541547556214</v>
-      </c>
-      <c r="M11" s="34">
-        <v>1.68</v>
-      </c>
-      <c r="N11" s="42">
-        <f t="shared" si="5"/>
-        <v>1.6455696202531647</v>
-      </c>
-      <c r="O11" s="32"/>
-      <c r="P11" s="38">
-        <f t="shared" si="6"/>
-        <v>19.59462128694738</v>
-      </c>
-      <c r="Q11" s="38">
-        <f t="shared" ref="Q11:Q19" si="7">$Q$4*$C11</f>
-        <v>75.707803029664063</v>
-      </c>
-      <c r="R11">
-        <f t="shared" ref="R11:R19" si="8">P11/4.448</f>
-        <v>4.4052655771014786</v>
-      </c>
-      <c r="S11" s="40">
-        <f t="shared" ref="S11:S19" si="9">Q11/4.448</f>
-        <v>17.020639170338143</v>
-      </c>
-      <c r="T11" s="34"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C11)*0.85</f>
+        <v>77.714970931527219</v>
+      </c>
+      <c r="Q11" s="57">
+        <f>($Q$4*$C11)*0.85</f>
+        <v>155.42994186305447</v>
+      </c>
+      <c r="R11" s="57">
+        <f t="shared" ref="R11:R19" si="5">P11/4.448</f>
+        <v>17.471890946836155</v>
+      </c>
+      <c r="S11" s="68">
+        <f t="shared" ref="S11:S19" si="6">Q11/4.448</f>
+        <v>34.943781893672316</v>
+      </c>
+      <c r="T11" s="66"/>
       <c r="U11" s="35"/>
       <c r="V11" s="39"/>
       <c r="W11" s="32"/>
@@ -5171,66 +5264,66 @@
       <c r="AK11" s="35"/>
       <c r="AL11" s="39"/>
     </row>
-    <row r="12" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B12" s="55">
         <v>0.6</v>
       </c>
       <c r="C12" s="57">
+        <f>$N$4*((1+(($O$4-1)/2)*($B12^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>27915.420137720866</v>
+      </c>
+      <c r="D12" s="57">
+        <v>0.47</v>
+      </c>
+      <c r="E12" s="35">
+        <v>1.68</v>
+      </c>
+      <c r="F12" s="68">
         <f t="shared" si="0"/>
-        <v>15760.414204094275</v>
-      </c>
-      <c r="D12" s="34">
-        <v>0.53300000000000003</v>
-      </c>
-      <c r="E12" s="34">
+        <v>1.6455696202531647</v>
+      </c>
+      <c r="G12" s="10"/>
+      <c r="H12" s="35">
+        <f t="shared" si="1"/>
+        <v>0.83757177792156701</v>
+      </c>
+      <c r="I12" s="35">
         <v>1.68</v>
       </c>
-      <c r="F12" s="39">
-        <f t="shared" si="1"/>
+      <c r="J12" s="68">
+        <f t="shared" si="2"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G12" s="32"/>
-      <c r="H12" s="34">
-        <f t="shared" si="2"/>
-        <v>0.61177588118659387</v>
-      </c>
-      <c r="I12" s="34">
+      <c r="K12" s="10"/>
+      <c r="L12" s="35">
+        <f t="shared" si="3"/>
+        <v>1.2051435558431343</v>
+      </c>
+      <c r="M12" s="35">
         <v>1.68</v>
       </c>
-      <c r="J12" s="39">
-        <f t="shared" si="3"/>
+      <c r="N12" s="68">
+        <f t="shared" si="4"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K12" s="32"/>
-      <c r="L12" s="34">
-        <f t="shared" si="4"/>
-        <v>0.83736663250724042</v>
-      </c>
-      <c r="M12" s="34">
-        <v>1.68</v>
-      </c>
-      <c r="N12" s="42">
+      <c r="O12" s="10"/>
+      <c r="P12" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C12)*0.85</f>
+        <v>183.70147445467921</v>
+      </c>
+      <c r="Q12" s="57">
+        <f>($Q$4*$C12)*0.85</f>
+        <v>367.40294890935849</v>
+      </c>
+      <c r="R12" s="57">
         <f t="shared" si="5"/>
-        <v>1.6455696202531647</v>
-      </c>
-      <c r="O12" s="32"/>
-      <c r="P12" s="38">
+        <v>41.299791918767802</v>
+      </c>
+      <c r="S12" s="68">
         <f t="shared" si="6"/>
-        <v>46.317469834284111</v>
-      </c>
-      <c r="Q12" s="38">
-        <f t="shared" si="7"/>
-        <v>178.95696128519953</v>
-      </c>
-      <c r="R12">
-        <f t="shared" si="8"/>
-        <v>10.413100232527901</v>
-      </c>
-      <c r="S12" s="40">
-        <f t="shared" si="9"/>
-        <v>40.233129785341617</v>
-      </c>
-      <c r="T12" s="34"/>
+        <v>82.599583837535619</v>
+      </c>
+      <c r="T12" s="66"/>
       <c r="U12" s="35"/>
       <c r="V12" s="39"/>
       <c r="W12" s="32"/>
@@ -5250,66 +5343,66 @@
       <c r="AK12" s="35"/>
       <c r="AL12" s="39"/>
     </row>
-    <row r="13" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B13" s="55">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="C13" s="57">
+        <f>$N$4*((1+(($O$4-1)/2)*($B13^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>70046.287909620587</v>
+      </c>
+      <c r="D13" s="57">
+        <v>0.47</v>
+      </c>
+      <c r="E13" s="35">
+        <v>1.68</v>
+      </c>
+      <c r="F13" s="68">
         <f t="shared" si="0"/>
-        <v>29995.29024315015</v>
-      </c>
-      <c r="D13" s="34">
-        <v>0.54800000000000004</v>
-      </c>
-      <c r="E13" s="34">
+        <v>1.6455696202531647</v>
+      </c>
+      <c r="G13" s="10"/>
+      <c r="H13" s="35">
+        <f t="shared" si="1"/>
+        <v>0.87992140555247178</v>
+      </c>
+      <c r="I13" s="35">
         <v>1.68</v>
       </c>
-      <c r="F13" s="39">
-        <f t="shared" si="1"/>
+      <c r="J13" s="68">
+        <f t="shared" si="2"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G13" s="32"/>
-      <c r="H13" s="34">
-        <f t="shared" si="2"/>
-        <v>0.63233371621683643</v>
-      </c>
-      <c r="I13" s="34">
+      <c r="K13" s="10"/>
+      <c r="L13" s="35">
+        <f t="shared" si="3"/>
+        <v>1.2898428111049438</v>
+      </c>
+      <c r="M13" s="35">
         <v>1.68</v>
       </c>
-      <c r="J13" s="39">
-        <f t="shared" si="3"/>
+      <c r="N13" s="68">
+        <f t="shared" si="4"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K13" s="32"/>
-      <c r="L13" s="34">
-        <f t="shared" si="4"/>
-        <v>0.87384045808310185</v>
-      </c>
-      <c r="M13" s="34">
-        <v>1.68</v>
-      </c>
-      <c r="N13" s="42">
+      <c r="O13" s="10"/>
+      <c r="P13" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C13)*0.85</f>
+        <v>460.94976559879348</v>
+      </c>
+      <c r="Q13" s="57">
+        <f>($Q$4*$C13)*0.85</f>
+        <v>921.89953119758695</v>
+      </c>
+      <c r="R13" s="57">
         <f t="shared" si="5"/>
-        <v>1.6455696202531647</v>
-      </c>
-      <c r="O13" s="32"/>
-      <c r="P13" s="38">
+        <v>103.63079262562802</v>
+      </c>
+      <c r="S13" s="68">
         <f t="shared" si="6"/>
-        <v>88.151614102044775</v>
-      </c>
-      <c r="Q13" s="38">
-        <f t="shared" si="7"/>
-        <v>340.59168276093078</v>
-      </c>
-      <c r="R13">
-        <f t="shared" si="8"/>
-        <v>19.818258566107186</v>
-      </c>
-      <c r="S13" s="40">
-        <f t="shared" si="9"/>
-        <v>76.571871124309965</v>
-      </c>
-      <c r="T13" s="34"/>
+        <v>207.26158525125604</v>
+      </c>
+      <c r="T13" s="66"/>
       <c r="U13" s="35"/>
       <c r="V13" s="39"/>
       <c r="W13" s="32"/>
@@ -5329,66 +5422,66 @@
       <c r="AK13" s="35"/>
       <c r="AL13" s="39"/>
     </row>
-    <row r="14" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B14" s="55">
         <v>1</v>
       </c>
       <c r="C14" s="57">
+        <f>$N$4*((1+(($O$4-1)/2)*($B14^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>90476.04700911307</v>
+      </c>
+      <c r="D14" s="57">
+        <v>0.63</v>
+      </c>
+      <c r="E14" s="35">
+        <v>1.68</v>
+      </c>
+      <c r="F14" s="68">
         <f t="shared" si="0"/>
-        <v>51080.727761855094</v>
-      </c>
-      <c r="D14" s="34">
-        <v>0.67200000000000004</v>
-      </c>
-      <c r="E14" s="34">
+        <v>1.6455696202531647</v>
+      </c>
+      <c r="G14" s="10"/>
+      <c r="H14" s="35">
+        <f t="shared" si="1"/>
+        <v>1.0588783355571327</v>
+      </c>
+      <c r="I14" s="35">
         <v>1.68</v>
       </c>
-      <c r="F14" s="39">
-        <f t="shared" si="1"/>
+      <c r="J14" s="68">
+        <f t="shared" si="2"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G14" s="32"/>
-      <c r="H14" s="34">
-        <f t="shared" si="2"/>
-        <v>0.76391475198773817</v>
-      </c>
-      <c r="I14" s="34">
+      <c r="K14" s="10"/>
+      <c r="L14" s="35">
+        <f t="shared" si="3"/>
+        <v>1.4877566711142658</v>
+      </c>
+      <c r="M14" s="35">
         <v>1.68</v>
       </c>
-      <c r="J14" s="39">
-        <f t="shared" si="3"/>
+      <c r="N14" s="68">
+        <f t="shared" si="4"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K14" s="32"/>
-      <c r="L14" s="34">
-        <f t="shared" si="4"/>
-        <v>1.0271313310476431</v>
-      </c>
-      <c r="M14" s="34">
-        <v>1.68</v>
-      </c>
-      <c r="N14" s="42">
+      <c r="O14" s="10"/>
+      <c r="P14" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C14)*0.85</f>
+        <v>595.39076096319559</v>
+      </c>
+      <c r="Q14" s="57">
+        <f>($Q$4*$C14)*0.85</f>
+        <v>1190.7815219263914</v>
+      </c>
+      <c r="R14" s="57">
         <f t="shared" si="5"/>
-        <v>1.6455696202531647</v>
-      </c>
-      <c r="O14" s="32"/>
-      <c r="P14" s="38">
+        <v>133.855836547481</v>
+      </c>
+      <c r="S14" s="68">
         <f t="shared" si="6"/>
-        <v>150.11852078153987</v>
-      </c>
-      <c r="Q14" s="38">
-        <f t="shared" si="7"/>
-        <v>580.01342490880631</v>
-      </c>
-      <c r="R14">
-        <f t="shared" si="8"/>
-        <v>33.749667441892953</v>
-      </c>
-      <c r="S14" s="40">
-        <f t="shared" si="9"/>
-        <v>130.39870164316687</v>
-      </c>
-      <c r="T14" s="34"/>
+        <v>267.71167309496207</v>
+      </c>
+      <c r="T14" s="66"/>
       <c r="U14" s="35"/>
       <c r="V14" s="39"/>
       <c r="W14" s="32"/>
@@ -5412,62 +5505,62 @@
       <c r="B15" s="56">
         <v>1.2</v>
       </c>
-      <c r="C15" s="58">
+      <c r="C15" s="57">
+        <f>$N$4*((1+(($O$4-1)/2)*($B15^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>144384.60456995908</v>
+      </c>
+      <c r="D15" s="57">
+        <v>0.6</v>
+      </c>
+      <c r="E15" s="35">
+        <v>1.68</v>
+      </c>
+      <c r="F15" s="68">
         <f t="shared" si="0"/>
-        <v>81516.278869901493</v>
-      </c>
-      <c r="D15" s="36">
-        <v>0.70299999999999996</v>
-      </c>
-      <c r="E15" s="17">
+        <v>1.6455696202531647</v>
+      </c>
+      <c r="G15" s="10"/>
+      <c r="H15" s="35">
+        <f t="shared" si="1"/>
+        <v>1.0752902297767035</v>
+      </c>
+      <c r="I15" s="35">
         <v>1.68</v>
       </c>
-      <c r="F15" s="41">
-        <f t="shared" si="1"/>
+      <c r="J15" s="68">
+        <f t="shared" si="2"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34">
-        <f t="shared" si="2"/>
-        <v>0.80486148371278865</v>
-      </c>
-      <c r="I15" s="34">
+      <c r="K15" s="10"/>
+      <c r="L15" s="35">
+        <f t="shared" si="3"/>
+        <v>1.5505804595534074</v>
+      </c>
+      <c r="M15" s="35">
         <v>1.68</v>
       </c>
-      <c r="J15" s="41">
-        <f t="shared" si="3"/>
+      <c r="N15" s="68">
+        <f t="shared" si="4"/>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K15" s="33"/>
-      <c r="L15" s="34">
-        <f t="shared" si="4"/>
-        <v>1.0965625512892234</v>
-      </c>
-      <c r="M15" s="34">
-        <v>1.68</v>
-      </c>
-      <c r="N15" s="51">
+      <c r="O15" s="10"/>
+      <c r="P15" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C15)*0.85</f>
+        <v>950.14384942811773</v>
+      </c>
+      <c r="Q15" s="57">
+        <f>($Q$4*$C15)*0.85</f>
+        <v>1900.2876988562355</v>
+      </c>
+      <c r="R15" s="57">
         <f t="shared" si="5"/>
-        <v>1.6455696202531647</v>
-      </c>
-      <c r="O15" s="33"/>
-      <c r="P15" s="38">
+        <v>213.61147693977466</v>
+      </c>
+      <c r="S15" s="68">
         <f t="shared" si="6"/>
-        <v>239.56399487133484</v>
-      </c>
-      <c r="Q15" s="38">
-        <f t="shared" si="7"/>
-        <v>925.604198780817</v>
-      </c>
-      <c r="R15">
-        <f t="shared" si="8"/>
-        <v>53.858811796613047</v>
-      </c>
-      <c r="S15" s="40">
-        <f t="shared" si="9"/>
-        <v>208.09446915036352</v>
-      </c>
-      <c r="T15" s="36"/>
+        <v>427.22295387954932</v>
+      </c>
+      <c r="T15" s="67"/>
       <c r="U15" s="17"/>
       <c r="V15" s="41"/>
       <c r="W15" s="33"/>
@@ -5487,184 +5580,184 @@
       <c r="AK15" s="17"/>
       <c r="AL15" s="41"/>
     </row>
-    <row r="16" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B16" s="55">
         <v>1.4</v>
       </c>
       <c r="C16" s="57">
-        <f t="shared" si="0"/>
-        <v>124838.62860986774</v>
-      </c>
-      <c r="D16" s="34">
-        <v>0.70599999999999996</v>
-      </c>
-      <c r="E16" s="34">
+        <f>$N$4*((1+(($O$4-1)/2)*($B16^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>221118.72961790801</v>
+      </c>
+      <c r="D16" s="57">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="E16" s="35">
         <v>1.68</v>
       </c>
-      <c r="F16" s="39">
+      <c r="F16" s="68">
         <f>(E16-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G16" s="32"/>
-      <c r="H16" s="34">
-        <f t="shared" si="2"/>
-        <v>0.8206096170322128</v>
-      </c>
-      <c r="I16" s="34">
+      <c r="G16" s="10"/>
+      <c r="H16" s="35">
+        <f t="shared" si="1"/>
+        <v>1.094773588881284</v>
+      </c>
+      <c r="I16" s="35">
         <v>1.68</v>
       </c>
-      <c r="J16" s="39">
+      <c r="J16" s="68">
         <f>(I16-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K16" s="32"/>
-      <c r="L16" s="34">
-        <f t="shared" si="4"/>
-        <v>1.1488175561300551</v>
-      </c>
-      <c r="M16" s="34">
+      <c r="K16" s="10"/>
+      <c r="L16" s="35">
+        <f t="shared" si="3"/>
+        <v>1.6295471777625679</v>
+      </c>
+      <c r="M16" s="35">
         <v>1.68</v>
       </c>
-      <c r="N16" s="42">
+      <c r="N16" s="68">
         <f>(M16-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="O16" s="32"/>
-      <c r="P16" s="38">
+      <c r="O16" s="10"/>
+      <c r="P16" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C16)*0.85</f>
+        <v>1455.1038981307493</v>
+      </c>
+      <c r="Q16" s="57">
+        <f>($Q$4*$C16)*0.85</f>
+        <v>2910.207796261499</v>
+      </c>
+      <c r="R16" s="57">
+        <f t="shared" si="5"/>
+        <v>327.13666774522238</v>
+      </c>
+      <c r="S16" s="68">
         <f t="shared" si="6"/>
-        <v>366.88181794669021</v>
-      </c>
-      <c r="Q16" s="38">
-        <f t="shared" si="7"/>
-        <v>1417.5224926023693</v>
-      </c>
-      <c r="R16">
-        <f t="shared" si="8"/>
-        <v>82.482423099525661</v>
-      </c>
-      <c r="S16" s="40">
-        <f t="shared" si="9"/>
-        <v>318.68761074693549</v>
+        <v>654.27333549044488</v>
       </c>
     </row>
-    <row r="17" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B17" s="55">
         <v>1.6</v>
       </c>
       <c r="C17" s="57">
-        <f t="shared" si="0"/>
-        <v>185942.55643692036</v>
-      </c>
-      <c r="D17" s="34">
-        <v>0.74399999999999999</v>
-      </c>
-      <c r="E17" s="34">
+        <f>$N$4*((1+(($O$4-1)/2)*($B17^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>329348.23394870316</v>
+      </c>
+      <c r="D17" s="57">
+        <v>0.5</v>
+      </c>
+      <c r="E17" s="35">
         <v>1.68</v>
       </c>
-      <c r="F17" s="39">
+      <c r="F17" s="68">
         <f>(E17-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G17" s="32"/>
-      <c r="H17" s="34">
-        <f t="shared" si="2"/>
-        <v>0.87469740832700682</v>
-      </c>
-      <c r="I17" s="34">
+      <c r="G17" s="10"/>
+      <c r="H17" s="35">
+        <f t="shared" si="1"/>
+        <v>1.1098399411706557</v>
+      </c>
+      <c r="I17" s="35">
         <v>1.68</v>
       </c>
-      <c r="J17" s="39">
+      <c r="J17" s="68">
         <f>(I17-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K17" s="32"/>
-      <c r="L17" s="34">
-        <f t="shared" si="4"/>
-        <v>1.2489760085284154</v>
-      </c>
-      <c r="M17" s="34">
+      <c r="K17" s="10"/>
+      <c r="L17" s="35">
+        <f t="shared" si="3"/>
+        <v>1.7196798823413117</v>
+      </c>
+      <c r="M17" s="35">
         <v>1.68</v>
       </c>
-      <c r="N17" s="42">
+      <c r="N17" s="68">
         <f>(M17-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="O17" s="32"/>
-      <c r="P17" s="38">
+      <c r="O17" s="10"/>
+      <c r="P17" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C17)*0.85</f>
+        <v>2167.3238621140463</v>
+      </c>
+      <c r="Q17" s="57">
+        <f>($Q$4*$C17)*0.85</f>
+        <v>4334.6477242280935</v>
+      </c>
+      <c r="R17" s="57">
+        <f t="shared" si="5"/>
+        <v>487.25806252563984</v>
+      </c>
+      <c r="S17" s="68">
         <f t="shared" si="6"/>
-        <v>546.45700532663568</v>
-      </c>
-      <c r="Q17" s="38">
-        <f t="shared" si="7"/>
-        <v>2111.3477376063215</v>
-      </c>
-      <c r="R17">
-        <f t="shared" si="8"/>
-        <v>122.85454256444146</v>
-      </c>
-      <c r="S17" s="40">
-        <f t="shared" si="9"/>
-        <v>474.67350215969452</v>
+        <v>974.51612505127991</v>
       </c>
     </row>
-    <row r="18" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B18" s="55">
         <v>1.8</v>
       </c>
       <c r="C18" s="57">
-        <f t="shared" si="0"/>
-        <v>271487.07906128647</v>
-      </c>
-      <c r="D18" s="34">
-        <v>0.68899999999999995</v>
-      </c>
-      <c r="E18" s="34">
+        <f>$N$4*((1+(($O$4-1)/2)*($B18^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>480867.81069431838</v>
+      </c>
+      <c r="D18" s="57">
+        <v>0.45</v>
+      </c>
+      <c r="E18" s="35">
         <v>1.68</v>
       </c>
-      <c r="F18" s="39">
+      <c r="F18" s="68">
         <f>(E18-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G18" s="32"/>
-      <c r="H18" s="34">
-        <f t="shared" si="2"/>
-        <v>0.83977602802731355</v>
-      </c>
-      <c r="I18" s="34">
+      <c r="G18" s="10"/>
+      <c r="H18" s="35">
+        <f t="shared" si="1"/>
+        <v>1.1535276769380436</v>
+      </c>
+      <c r="I18" s="35">
         <v>1.68</v>
       </c>
-      <c r="J18" s="39">
+      <c r="J18" s="68">
         <f>(I18-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K18" s="32"/>
-      <c r="L18" s="34">
-        <f t="shared" si="4"/>
-        <v>1.2715538378274662</v>
-      </c>
-      <c r="M18" s="34">
+      <c r="K18" s="10"/>
+      <c r="L18" s="35">
+        <f t="shared" si="3"/>
+        <v>1.8570553538760872</v>
+      </c>
+      <c r="M18" s="35">
         <v>1.68</v>
       </c>
-      <c r="N18" s="42">
+      <c r="N18" s="68">
         <f>(M18-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="O18" s="32"/>
-      <c r="P18" s="38">
+      <c r="O18" s="10"/>
+      <c r="P18" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C18)*0.85</f>
+        <v>3164.420431665837</v>
+      </c>
+      <c r="Q18" s="57">
+        <f>($Q$4*$C18)*0.85</f>
+        <v>6328.840863331674</v>
+      </c>
+      <c r="R18" s="57">
+        <f t="shared" si="5"/>
+        <v>711.42545675940573</v>
+      </c>
+      <c r="S18" s="68">
         <f t="shared" si="6"/>
-        <v>797.85939836228329</v>
-      </c>
-      <c r="Q18" s="38">
-        <f t="shared" si="7"/>
-        <v>3082.6919945023496</v>
-      </c>
-      <c r="R18">
-        <f t="shared" si="8"/>
-        <v>179.37486473972194</v>
-      </c>
-      <c r="S18" s="40">
-        <f t="shared" si="9"/>
-        <v>693.05125775682313</v>
+        <v>1422.8509135188115</v>
       </c>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.25">
@@ -5672,68 +5765,73 @@
         <v>2</v>
       </c>
       <c r="C19" s="57">
-        <f t="shared" si="0"/>
-        <v>390398.07525384444</v>
-      </c>
-      <c r="D19" s="34">
-        <v>0.64400000000000002</v>
-      </c>
-      <c r="E19" s="34">
+        <f>$N$4*((1+(($O$4-1)/2)*($B19^2))^($O$4/($O$4-1))) - $N$4</f>
+        <v>691487.30170032557</v>
+      </c>
+      <c r="D19" s="57">
+        <v>0.4</v>
+      </c>
+      <c r="E19" s="35">
         <v>1.68</v>
       </c>
-      <c r="F19" s="39">
+      <c r="F19" s="68">
         <f>(E19-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="G19" s="32"/>
-      <c r="H19" s="34">
-        <f t="shared" si="2"/>
-        <v>0.81962074698083875</v>
-      </c>
-      <c r="I19" s="34">
+      <c r="G19" s="10"/>
+      <c r="H19" s="35">
+        <f t="shared" si="1"/>
+        <v>1.2194542445644689</v>
+      </c>
+      <c r="I19" s="35">
         <v>1.68</v>
       </c>
-      <c r="J19" s="39">
+      <c r="J19" s="68">
         <f>(I19-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="K19" s="32"/>
-      <c r="L19" s="34">
-        <f t="shared" si="4"/>
-        <v>1.3225464605638804</v>
-      </c>
-      <c r="M19" s="34">
+      <c r="K19" s="10"/>
+      <c r="L19" s="35">
+        <f t="shared" si="3"/>
+        <v>2.0389084891289384</v>
+      </c>
+      <c r="M19" s="35">
         <v>1.68</v>
       </c>
-      <c r="N19" s="42">
+      <c r="N19" s="68">
         <f>(M19-$M$4)/$L$4</f>
         <v>1.6455696202531647</v>
       </c>
-      <c r="O19" s="32"/>
-      <c r="P19" s="38">
+      <c r="O19" s="10"/>
+      <c r="P19" s="57">
+        <f>($Q$4*SIN(RADIANS($G$10))*C19)*0.85</f>
+        <v>4550.4325660279483</v>
+      </c>
+      <c r="Q19" s="57">
+        <f>($Q$4*$C19)*0.85</f>
+        <v>9100.8651320558965</v>
+      </c>
+      <c r="R19" s="57">
+        <f t="shared" si="5"/>
+        <v>1023.0289042329019</v>
+      </c>
+      <c r="S19" s="68">
         <f t="shared" si="6"/>
-        <v>1147.3208025988981</v>
-      </c>
-      <c r="Q19" s="38">
-        <f t="shared" si="7"/>
-        <v>4432.907177075911</v>
-      </c>
-      <c r="R19">
-        <f t="shared" si="8"/>
-        <v>257.94082792241414</v>
-      </c>
-      <c r="S19" s="40">
-        <f t="shared" si="9"/>
-        <v>996.606829378577</v>
+        <v>2046.0578084658039</v>
+      </c>
+    </row>
+    <row r="23" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="Q23">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="25" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="G25">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="J2:M2"/>
     <mergeCell ref="AI8:AL8"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="O8:R8"/>
@@ -5741,6 +5839,11 @@
     <mergeCell ref="W8:Z8"/>
     <mergeCell ref="AA8:AD8"/>
     <mergeCell ref="AE8:AH8"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="J2:M2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5766,21 +5869,21 @@
   <sheetData>
     <row r="1" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="61"/>
-      <c r="J2" s="64" t="s">
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="60"/>
+      <c r="J2" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="65"/>
-      <c r="L2" s="65"/>
-      <c r="M2" s="66"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="63"/>
     </row>
     <row r="3" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -5924,54 +6027,54 @@
       </c>
     </row>
     <row r="8" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="59" t="s">
+      <c r="C8" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="59" t="s">
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="60"/>
+      <c r="G8" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="60"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="59" t="s">
+      <c r="H8" s="59"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="60"/>
+      <c r="K8" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="L8" s="60"/>
-      <c r="M8" s="60"/>
-      <c r="N8" s="61"/>
-      <c r="O8" s="59"/>
-      <c r="P8" s="60"/>
-      <c r="Q8" s="60"/>
-      <c r="R8" s="61"/>
-      <c r="S8" s="59"/>
-      <c r="T8" s="60"/>
-      <c r="U8" s="60"/>
-      <c r="V8" s="61"/>
-      <c r="W8" s="59"/>
-      <c r="X8" s="60"/>
-      <c r="Y8" s="60"/>
-      <c r="Z8" s="61"/>
-      <c r="AA8" s="59"/>
-      <c r="AB8" s="60"/>
-      <c r="AC8" s="60"/>
-      <c r="AD8" s="61"/>
-      <c r="AE8" s="59"/>
-      <c r="AF8" s="60"/>
-      <c r="AG8" s="60"/>
-      <c r="AH8" s="61"/>
-      <c r="AI8" s="59"/>
-      <c r="AJ8" s="60"/>
-      <c r="AK8" s="60"/>
-      <c r="AL8" s="61"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
+      <c r="N8" s="60"/>
+      <c r="O8" s="58"/>
+      <c r="P8" s="59"/>
+      <c r="Q8" s="59"/>
+      <c r="R8" s="60"/>
+      <c r="S8" s="58"/>
+      <c r="T8" s="59"/>
+      <c r="U8" s="59"/>
+      <c r="V8" s="60"/>
+      <c r="W8" s="58"/>
+      <c r="X8" s="59"/>
+      <c r="Y8" s="59"/>
+      <c r="Z8" s="60"/>
+      <c r="AA8" s="58"/>
+      <c r="AB8" s="59"/>
+      <c r="AC8" s="59"/>
+      <c r="AD8" s="60"/>
+      <c r="AE8" s="58"/>
+      <c r="AF8" s="59"/>
+      <c r="AG8" s="59"/>
+      <c r="AH8" s="60"/>
+      <c r="AI8" s="58"/>
+      <c r="AJ8" s="59"/>
+      <c r="AK8" s="59"/>
+      <c r="AL8" s="60"/>
     </row>
     <row r="9" spans="2:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="63"/>
+      <c r="B9" s="65"/>
       <c r="C9" s="25" t="s">
         <v>13</v>
       </c>

</xml_diff>